<commit_message>
Add Pierce Lazer Cruiser, Make Cornuto 2 Taller
- yes I know it's misspelled.
- also edited fleet stats to correct the value (make it a whole number)
</commit_message>
<xml_diff>
--- a/! Other Assets/Fleet Statsv2.xlsx
+++ b/! Other Assets/Fleet Statsv2.xlsx
@@ -1,23 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ty\Documents\From The Depths\Player Profiles\Rhayader\Constructables\! Other Assets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14AA4F4-B24E-4AC9-A6F8-8CF59C3BF0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="31950" yWindow="1260" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Fleet Stats" sheetId="1" r:id="rId4"/>
+    <sheet name="Fleet Stats" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.2">'Fleet Stats'!$D$2:$D$37</definedName>
-    <definedName name="_xlchart.v1.4">'Fleet Stats'!$F$2:$F$37</definedName>
-    <definedName name="_xlchart.v1.6">'Fleet Stats'!$E$2:$E$37</definedName>
-    <definedName name="_xlchart.v1.3">'Fleet Stats'!$E$2:$E$37</definedName>
-    <definedName name="_xlchart.v1.7">'Fleet Stats'!$B$2:$B$37</definedName>
-    <definedName name="_xlchart.v1.8">'Fleet Stats'!$E$2:$E$37</definedName>
-    <definedName name="_xlchart.v1.0">'Fleet Stats'!$B$2:$B$37</definedName>
-    <definedName name="_xlchart.v1.5">'Fleet Stats'!$B$2:$B$37</definedName>
-    <definedName name="_xlchart.v1.1">'Fleet Stats'!$C$2:$C$37</definedName>
-  </definedNames>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="HYZ7l2qcTpMFmE/tPuZ0oH5AxGhRxXxzwEEuKCQp/yI="/>
     </ext>
@@ -232,30 +242,32 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -265,7 +277,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -329,167 +341,157 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="57">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="7" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="9" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="8" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="10" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="9" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="10" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="11" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="3" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="7" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="9" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="9" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="10" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="10" fontId="2" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="11" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="11" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="11" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -679,28 +681,28 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B1:R1000"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.63"/>
-    <col customWidth="1" min="2" max="2" width="17.13"/>
-    <col customWidth="1" min="3" max="7" width="14.25"/>
-    <col customWidth="1" min="8" max="8" width="8.63"/>
-    <col customWidth="1" min="9" max="9" width="17.13"/>
-    <col customWidth="1" min="10" max="14" width="14.25"/>
-    <col customWidth="1" min="15" max="15" width="8.63"/>
-    <col customWidth="1" min="16" max="16" width="15.0"/>
-    <col customWidth="1" min="17" max="26" width="8.63"/>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="10" max="14" width="14.28515625" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" customWidth="1"/>
+    <col min="16" max="16" width="15" customWidth="1"/>
+    <col min="17" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -744,18 +746,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="3">
-        <v>52498.0</v>
+        <v>52498</v>
       </c>
       <c r="D2" s="4">
-        <v>160632.0</v>
+        <v>160632</v>
       </c>
       <c r="E2" s="3">
-        <v>2468826.0</v>
+        <v>2468826</v>
       </c>
       <c r="F2" s="4">
         <v>718.5</v>
@@ -767,13 +769,13 @@
         <v>9</v>
       </c>
       <c r="J2" s="4">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="K2" s="4">
-        <v>152644.0</v>
+        <v>152644</v>
       </c>
       <c r="L2" s="4">
-        <v>3281122.0</v>
+        <v>3281122</v>
       </c>
       <c r="M2" s="4"/>
       <c r="N2" s="4" t="b">
@@ -789,18 +791,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="3">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="D3" s="4">
-        <v>152644.0</v>
+        <v>152644</v>
       </c>
       <c r="E3" s="5">
-        <v>1881122.0</v>
+        <v>1881122</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4" t="b">
@@ -810,13 +812,13 @@
         <v>8</v>
       </c>
       <c r="J3" s="4">
-        <v>52498.0</v>
+        <v>52498</v>
       </c>
       <c r="K3" s="4">
-        <v>160632.0</v>
+        <v>160632</v>
       </c>
       <c r="L3" s="4">
-        <v>2468826.0</v>
+        <v>2468826</v>
       </c>
       <c r="M3" s="4">
         <v>718.5</v>
@@ -834,18 +836,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="3">
-        <v>39723.0</v>
+        <v>39723</v>
       </c>
       <c r="D4" s="4">
-        <v>129765.0</v>
+        <v>129765</v>
       </c>
       <c r="E4" s="3">
-        <v>1725148.0</v>
+        <v>1725148</v>
       </c>
       <c r="F4" s="4">
         <v>1386.36</v>
@@ -857,13 +859,13 @@
         <v>12</v>
       </c>
       <c r="J4" s="4">
-        <v>25421.0</v>
+        <v>25421</v>
       </c>
       <c r="K4" s="4">
-        <v>76292.0</v>
+        <v>76292</v>
       </c>
       <c r="L4" s="4">
-        <v>1976556.0</v>
+        <v>1976556</v>
       </c>
       <c r="M4" s="4">
         <v>358.28</v>
@@ -881,18 +883,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="4">
-        <v>30502.0</v>
+        <v>30502</v>
       </c>
       <c r="D5" s="4">
-        <v>78691.0</v>
+        <v>78691</v>
       </c>
       <c r="E5" s="6">
-        <v>968078.0</v>
+        <v>968078</v>
       </c>
       <c r="F5" s="4">
         <v>458.24</v>
@@ -904,13 +906,13 @@
         <v>11</v>
       </c>
       <c r="J5" s="4">
-        <v>39723.0</v>
+        <v>39723</v>
       </c>
       <c r="K5" s="4">
-        <v>129765.0</v>
+        <v>129765</v>
       </c>
       <c r="L5" s="4">
-        <v>1725148.0</v>
+        <v>1725148</v>
       </c>
       <c r="M5" s="4">
         <v>1386.36</v>
@@ -928,21 +930,21 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="3">
-        <v>24173.0</v>
+        <v>24173</v>
       </c>
       <c r="D6" s="4">
-        <v>77248.0</v>
+        <v>77248</v>
       </c>
       <c r="E6" s="3">
-        <v>1283686.0</v>
+        <v>1283686</v>
       </c>
       <c r="F6" s="4">
-        <v>1026.64</v>
+        <v>1026.6400000000001</v>
       </c>
       <c r="G6" s="4" t="b">
         <v>0</v>
@@ -951,13 +953,13 @@
         <v>15</v>
       </c>
       <c r="J6" s="4">
-        <v>24137.0</v>
+        <v>24137</v>
       </c>
       <c r="K6" s="4">
-        <v>73293.0</v>
+        <v>73293</v>
       </c>
       <c r="L6" s="4">
-        <v>1588139.0</v>
+        <v>1588139</v>
       </c>
       <c r="M6" s="4"/>
       <c r="N6" s="4" t="b">
@@ -973,18 +975,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="3">
-        <v>25421.0</v>
+        <v>25421</v>
       </c>
       <c r="D7" s="4">
-        <v>76292.0</v>
+        <v>76292</v>
       </c>
       <c r="E7" s="3">
-        <v>1976556.0</v>
+        <v>1976556</v>
       </c>
       <c r="F7" s="4">
         <v>358.28</v>
@@ -996,16 +998,16 @@
         <v>14</v>
       </c>
       <c r="J7" s="4">
-        <v>24173.0</v>
+        <v>24173</v>
       </c>
       <c r="K7" s="4">
-        <v>77248.0</v>
+        <v>77248</v>
       </c>
       <c r="L7" s="4">
-        <v>1283686.0</v>
+        <v>1283686</v>
       </c>
       <c r="M7" s="4">
-        <v>1026.64</v>
+        <v>1026.6400000000001</v>
       </c>
       <c r="N7" s="4" t="b">
         <v>0</v>
@@ -1020,18 +1022,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="3">
-        <v>23500.0</v>
+        <v>23500</v>
       </c>
       <c r="D8" s="4">
-        <v>73787.0</v>
+        <v>73787</v>
       </c>
       <c r="E8" s="3">
-        <v>928002.0</v>
+        <v>928002</v>
       </c>
       <c r="F8" s="4">
         <v>852.28</v>
@@ -1043,13 +1045,13 @@
         <v>13</v>
       </c>
       <c r="J8" s="4">
-        <v>30502.0</v>
+        <v>30502</v>
       </c>
       <c r="K8" s="4">
-        <v>78691.0</v>
+        <v>78691</v>
       </c>
       <c r="L8" s="4">
-        <v>968078.0</v>
+        <v>968078</v>
       </c>
       <c r="M8" s="4">
         <v>458.24</v>
@@ -1067,18 +1069,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="3">
-        <v>24137.0</v>
+        <v>24137</v>
       </c>
       <c r="D9" s="4">
-        <v>73293.0</v>
+        <v>73293</v>
       </c>
       <c r="E9" s="3">
-        <v>1588139.0</v>
+        <v>1588139</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="b">
@@ -1088,13 +1090,13 @@
         <v>16</v>
       </c>
       <c r="J9" s="4">
-        <v>23500.0</v>
+        <v>23500</v>
       </c>
       <c r="K9" s="4">
-        <v>73787.0</v>
+        <v>73787</v>
       </c>
       <c r="L9" s="4">
-        <v>928002.0</v>
+        <v>928002</v>
       </c>
       <c r="M9" s="4">
         <v>852.28</v>
@@ -1112,18 +1114,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="8">
-        <v>26378.0</v>
+        <v>26378</v>
       </c>
       <c r="D10" s="9">
-        <v>68221.0</v>
+        <v>68221</v>
       </c>
       <c r="E10" s="8">
-        <v>671137.0</v>
+        <v>671137</v>
       </c>
       <c r="F10" s="9">
         <v>616.59</v>
@@ -1135,13 +1137,13 @@
         <v>18</v>
       </c>
       <c r="J10" s="4">
-        <v>23368.0</v>
+        <v>23368</v>
       </c>
       <c r="K10" s="4">
-        <v>67046.0</v>
+        <v>67046</v>
       </c>
       <c r="L10" s="4">
-        <v>872971.0</v>
+        <v>872971</v>
       </c>
       <c r="M10" s="4">
         <v>367.2</v>
@@ -1159,18 +1161,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="3">
-        <v>23368.0</v>
+        <v>23368</v>
       </c>
       <c r="D11" s="4">
-        <v>67046.0</v>
+        <v>67046</v>
       </c>
       <c r="E11" s="3">
-        <v>872971.0</v>
+        <v>872971</v>
       </c>
       <c r="F11" s="4">
         <v>367.2</v>
@@ -1182,13 +1184,13 @@
         <v>20</v>
       </c>
       <c r="J11" s="10">
-        <v>6248.0</v>
+        <v>6248</v>
       </c>
       <c r="K11" s="10">
-        <v>16591.0</v>
+        <v>16591</v>
       </c>
       <c r="L11" s="10">
-        <v>708732.0</v>
+        <v>708732</v>
       </c>
       <c r="M11" s="10">
         <v>327.71</v>
@@ -1206,18 +1208,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="3">
-        <v>15053.0</v>
+        <v>15053</v>
       </c>
       <c r="D12" s="4">
-        <v>50834.0</v>
+        <v>50834</v>
       </c>
       <c r="E12" s="3">
-        <v>320017.0</v>
+        <v>320017</v>
       </c>
       <c r="F12" s="4">
         <v>204.44</v>
@@ -1229,13 +1231,13 @@
         <v>17</v>
       </c>
       <c r="J12" s="10">
-        <v>26378.0</v>
+        <v>26378</v>
       </c>
       <c r="K12" s="10">
-        <v>68221.0</v>
+        <v>68221</v>
       </c>
       <c r="L12" s="10">
-        <v>671137.0</v>
+        <v>671137</v>
       </c>
       <c r="M12" s="10">
         <v>616.59</v>
@@ -1253,18 +1255,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="12">
-        <v>16938.0</v>
+        <v>16938</v>
       </c>
       <c r="D13" s="10">
-        <v>37667.0</v>
+        <v>37667</v>
       </c>
       <c r="E13" s="12">
-        <v>492176.0</v>
+        <v>492176</v>
       </c>
       <c r="F13" s="10">
         <v>805.25</v>
@@ -1276,13 +1278,13 @@
         <v>24</v>
       </c>
       <c r="J13" s="13">
-        <v>16938.0</v>
+        <v>16938</v>
       </c>
       <c r="K13" s="13">
-        <v>37667.0</v>
+        <v>37667</v>
       </c>
       <c r="L13" s="13">
-        <v>492176.0</v>
+        <v>492176</v>
       </c>
       <c r="M13" s="13">
         <v>805.25</v>
@@ -1300,18 +1302,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C14" s="12">
-        <v>13756.0</v>
+        <v>13756</v>
       </c>
       <c r="D14" s="10">
-        <v>36776.0</v>
+        <v>36776</v>
       </c>
       <c r="E14" s="12">
-        <v>486956.0</v>
+        <v>486956</v>
       </c>
       <c r="F14" s="10">
         <v>449.04</v>
@@ -1323,13 +1325,13 @@
         <v>25</v>
       </c>
       <c r="J14" s="13">
-        <v>13756.0</v>
+        <v>13756</v>
       </c>
       <c r="K14" s="13">
-        <v>36776.0</v>
+        <v>36776</v>
       </c>
       <c r="L14" s="13">
-        <v>486956.0</v>
+        <v>486956</v>
       </c>
       <c r="M14" s="13">
         <v>449.04</v>
@@ -1347,18 +1349,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C15" s="14">
-        <v>11135.0</v>
+        <v>11135</v>
       </c>
       <c r="D15" s="10">
-        <v>34940.0</v>
+        <v>34940</v>
       </c>
       <c r="E15" s="14">
-        <v>341813.0</v>
+        <v>341813</v>
       </c>
       <c r="F15" s="10">
         <v>172.87</v>
@@ -1370,13 +1372,13 @@
         <v>28</v>
       </c>
       <c r="J15" s="13">
-        <v>5575.0</v>
+        <v>5575</v>
       </c>
       <c r="K15" s="13">
-        <v>14906.0</v>
+        <v>14906</v>
       </c>
       <c r="L15" s="13">
-        <v>422837.0</v>
+        <v>422837</v>
       </c>
       <c r="M15" s="13">
         <v>112.08</v>
@@ -1394,21 +1396,21 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="16">
-        <v>9642.0</v>
+        <v>9642</v>
       </c>
       <c r="D16" s="13">
-        <v>28703.0</v>
+        <v>28703</v>
       </c>
       <c r="E16" s="16">
-        <v>402723.0</v>
+        <v>402723</v>
       </c>
       <c r="F16" s="13">
-        <v>524.45</v>
+        <v>524.45000000000005</v>
       </c>
       <c r="G16" s="13" t="b">
         <v>0</v>
@@ -1417,16 +1419,16 @@
         <v>29</v>
       </c>
       <c r="J16" s="13">
-        <v>9642.0</v>
+        <v>9642</v>
       </c>
       <c r="K16" s="13">
-        <v>28703.0</v>
+        <v>28703</v>
       </c>
       <c r="L16" s="13">
-        <v>402723.0</v>
+        <v>402723</v>
       </c>
       <c r="M16" s="13">
-        <v>524.45</v>
+        <v>524.45000000000005</v>
       </c>
       <c r="N16" s="13" t="b">
         <v>0</v>
@@ -1441,18 +1443,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" s="15" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="16">
-        <v>8255.0</v>
+        <v>8255</v>
       </c>
       <c r="D17" s="13">
-        <v>27268.0</v>
+        <v>27268</v>
       </c>
       <c r="E17" s="16">
-        <v>369225.0</v>
+        <v>369225</v>
       </c>
       <c r="F17" s="13">
         <v>219.44</v>
@@ -1464,13 +1466,13 @@
         <v>30</v>
       </c>
       <c r="J17" s="13">
-        <v>8255.0</v>
+        <v>8255</v>
       </c>
       <c r="K17" s="13">
-        <v>27268.0</v>
+        <v>27268</v>
       </c>
       <c r="L17" s="13">
-        <v>369225.0</v>
+        <v>369225</v>
       </c>
       <c r="M17" s="13">
         <v>219.44</v>
@@ -1488,18 +1490,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B18" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="16">
-        <v>9310.0</v>
+        <v>9310</v>
       </c>
       <c r="D18" s="13">
-        <v>26903.0</v>
+        <v>26903</v>
       </c>
       <c r="E18" s="16">
-        <v>354630.0</v>
+        <v>354630</v>
       </c>
       <c r="F18" s="13">
         <v>317.05</v>
@@ -1511,13 +1513,13 @@
         <v>32</v>
       </c>
       <c r="J18" s="13">
-        <v>9310.0</v>
+        <v>9310</v>
       </c>
       <c r="K18" s="13">
-        <v>26903.0</v>
+        <v>26903</v>
       </c>
       <c r="L18" s="13">
-        <v>354630.0</v>
+        <v>354630</v>
       </c>
       <c r="M18" s="13">
         <v>317.05</v>
@@ -1535,18 +1537,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B19" s="15" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="16">
-        <v>10667.0</v>
+        <v>10667</v>
       </c>
       <c r="D19" s="13">
-        <v>26278.0</v>
+        <v>26278</v>
       </c>
       <c r="E19" s="16">
-        <v>273866.0</v>
+        <v>273866</v>
       </c>
       <c r="F19" s="13">
         <v>402.63</v>
@@ -1558,13 +1560,13 @@
         <v>27</v>
       </c>
       <c r="J19" s="17">
-        <v>11135.0</v>
+        <v>11135</v>
       </c>
       <c r="K19" s="17">
-        <v>34940.0</v>
+        <v>34940</v>
       </c>
       <c r="L19" s="17">
-        <v>341813.0</v>
+        <v>341813</v>
       </c>
       <c r="M19" s="17">
         <v>172.87</v>
@@ -1582,18 +1584,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C20" s="16">
-        <v>8436.0</v>
+        <v>8436</v>
       </c>
       <c r="D20" s="13">
-        <v>26125.0</v>
+        <v>26125</v>
       </c>
       <c r="E20" s="16">
-        <v>340606.0</v>
+        <v>340606</v>
       </c>
       <c r="F20" s="13">
         <v>239.82</v>
@@ -1605,13 +1607,13 @@
         <v>34</v>
       </c>
       <c r="J20" s="17">
-        <v>8436.0</v>
+        <v>8436</v>
       </c>
       <c r="K20" s="17">
-        <v>26125.0</v>
+        <v>26125</v>
       </c>
       <c r="L20" s="17">
-        <v>340606.0</v>
+        <v>340606</v>
       </c>
       <c r="M20" s="17">
         <v>239.82</v>
@@ -1629,21 +1631,21 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C21" s="16">
-        <v>8403.0</v>
+        <v>8403</v>
       </c>
       <c r="D21" s="13">
-        <v>25428.0</v>
+        <v>25428</v>
       </c>
       <c r="E21" s="16">
-        <v>260829.0</v>
+        <v>260829</v>
       </c>
       <c r="F21" s="13">
-        <v>151.42</v>
+        <v>151.41999999999999</v>
       </c>
       <c r="G21" s="13" t="b">
         <v>0</v>
@@ -1652,13 +1654,13 @@
         <v>36</v>
       </c>
       <c r="J21" s="17">
-        <v>6161.0</v>
+        <v>6161</v>
       </c>
       <c r="K21" s="17">
-        <v>18678.0</v>
+        <v>18678</v>
       </c>
       <c r="L21" s="17">
-        <v>335199.0</v>
+        <v>335199</v>
       </c>
       <c r="M21" s="17">
         <v>158.46</v>
@@ -1676,18 +1678,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="17" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="18">
-        <v>6161.0</v>
+        <v>6161</v>
       </c>
       <c r="D22" s="17">
-        <v>18678.0</v>
+        <v>18678</v>
       </c>
       <c r="E22" s="18">
-        <v>335199.0</v>
+        <v>335199</v>
       </c>
       <c r="F22" s="17">
         <v>158.46</v>
@@ -1699,13 +1701,13 @@
         <v>22</v>
       </c>
       <c r="J22" s="17">
-        <v>15053.0</v>
+        <v>15053</v>
       </c>
       <c r="K22" s="17">
-        <v>50834.0</v>
+        <v>50834</v>
       </c>
       <c r="L22" s="17">
-        <v>320017.0</v>
+        <v>320017</v>
       </c>
       <c r="M22" s="17">
         <v>204.44</v>
@@ -1723,18 +1725,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="17" t="s">
         <v>37</v>
       </c>
       <c r="C23" s="18">
-        <v>5966.0</v>
+        <v>5966</v>
       </c>
       <c r="D23" s="17">
-        <v>17888.0</v>
+        <v>17888</v>
       </c>
       <c r="E23" s="18">
-        <v>176080.0</v>
+        <v>176080</v>
       </c>
       <c r="F23" s="17">
         <v>55.82</v>
@@ -1746,13 +1748,13 @@
         <v>33</v>
       </c>
       <c r="J23" s="17">
-        <v>10667.0</v>
+        <v>10667</v>
       </c>
       <c r="K23" s="17">
-        <v>26278.0</v>
+        <v>26278</v>
       </c>
       <c r="L23" s="17">
-        <v>273866.0</v>
+        <v>273866</v>
       </c>
       <c r="M23" s="17">
         <v>402.63</v>
@@ -1770,18 +1772,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="19" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="20">
-        <v>6248.0</v>
+        <v>6248</v>
       </c>
       <c r="D24" s="17">
-        <v>16591.0</v>
+        <v>16591</v>
       </c>
       <c r="E24" s="20">
-        <v>708732.0</v>
+        <v>708732</v>
       </c>
       <c r="F24" s="17">
         <v>327.71</v>
@@ -1793,16 +1795,16 @@
         <v>35</v>
       </c>
       <c r="J24" s="17">
-        <v>8403.0</v>
+        <v>8403</v>
       </c>
       <c r="K24" s="17">
-        <v>25428.0</v>
+        <v>25428</v>
       </c>
       <c r="L24" s="17">
-        <v>260829.0</v>
+        <v>260829</v>
       </c>
       <c r="M24" s="17">
-        <v>151.42</v>
+        <v>151.41999999999999</v>
       </c>
       <c r="N24" s="17" t="b">
         <v>0</v>
@@ -1817,18 +1819,18 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="17" t="s">
         <v>38</v>
       </c>
       <c r="C25" s="18">
-        <v>5531.0</v>
+        <v>5531</v>
       </c>
       <c r="D25" s="17">
-        <v>15365.0</v>
+        <v>15365</v>
       </c>
       <c r="E25" s="18">
-        <v>232077.0</v>
+        <v>232077</v>
       </c>
       <c r="F25" s="17">
         <v>118.01</v>
@@ -1840,13 +1842,13 @@
         <v>38</v>
       </c>
       <c r="J25" s="17">
-        <v>5531.0</v>
+        <v>5531</v>
       </c>
       <c r="K25" s="17">
-        <v>15365.0</v>
+        <v>15365</v>
       </c>
       <c r="L25" s="17">
-        <v>232077.0</v>
+        <v>232077</v>
       </c>
       <c r="M25" s="17">
         <v>118.01</v>
@@ -1864,18 +1866,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="17" t="s">
         <v>39</v>
       </c>
       <c r="C26" s="18">
-        <v>5371.0</v>
+        <v>5371</v>
       </c>
       <c r="D26" s="17">
-        <v>15001.0</v>
+        <v>15001</v>
       </c>
       <c r="E26" s="18">
-        <v>169596.0</v>
+        <v>169596</v>
       </c>
       <c r="F26" s="17">
         <v>77.03</v>
@@ -1887,13 +1889,13 @@
         <v>40</v>
       </c>
       <c r="J26" s="21">
-        <v>4594.0</v>
+        <v>4594</v>
       </c>
       <c r="K26" s="21">
-        <v>12337.0</v>
+        <v>12337</v>
       </c>
       <c r="L26" s="21">
-        <v>187586.0</v>
+        <v>187586</v>
       </c>
       <c r="M26" s="21">
         <v>98.01</v>
@@ -1911,18 +1913,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
         <v>28</v>
       </c>
       <c r="C27" s="22">
-        <v>5575.0</v>
+        <v>5575</v>
       </c>
       <c r="D27" s="21">
-        <v>14906.0</v>
+        <v>14906</v>
       </c>
       <c r="E27" s="22">
-        <v>422837.0</v>
+        <v>422837</v>
       </c>
       <c r="F27" s="21">
         <v>112.08</v>
@@ -1934,16 +1936,16 @@
         <v>41</v>
       </c>
       <c r="J27" s="21">
-        <v>4634.0</v>
+        <v>4634</v>
       </c>
       <c r="K27" s="21">
-        <v>12365.0</v>
+        <v>12365</v>
       </c>
       <c r="L27" s="21">
-        <v>179274.0</v>
+        <v>179274</v>
       </c>
       <c r="M27" s="21">
-        <v>80.85</v>
+        <v>80.849999999999994</v>
       </c>
       <c r="N27" s="21" t="b">
         <v>1</v>
@@ -1958,21 +1960,21 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="21" t="s">
         <v>41</v>
       </c>
       <c r="C28" s="22">
-        <v>4634.0</v>
+        <v>4634</v>
       </c>
       <c r="D28" s="21">
-        <v>12365.0</v>
+        <v>12365</v>
       </c>
       <c r="E28" s="22">
-        <v>179274.0</v>
+        <v>179274</v>
       </c>
       <c r="F28" s="21">
-        <v>80.85</v>
+        <v>80.849999999999994</v>
       </c>
       <c r="G28" s="21" t="b">
         <v>1</v>
@@ -1981,13 +1983,13 @@
         <v>37</v>
       </c>
       <c r="J28" s="21">
-        <v>5966.0</v>
+        <v>5966</v>
       </c>
       <c r="K28" s="21">
-        <v>17888.0</v>
+        <v>17888</v>
       </c>
       <c r="L28" s="21">
-        <v>176080.0</v>
+        <v>176080</v>
       </c>
       <c r="M28" s="21">
         <v>55.82</v>
@@ -2005,18 +2007,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="23" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="24">
-        <v>4594.0</v>
+        <v>4594</v>
       </c>
       <c r="D29" s="21">
-        <v>12337.0</v>
+        <v>12337</v>
       </c>
       <c r="E29" s="24">
-        <v>187586.0</v>
+        <v>187586</v>
       </c>
       <c r="F29" s="21">
         <v>98.01</v>
@@ -2028,13 +2030,13 @@
         <v>39</v>
       </c>
       <c r="J29" s="21">
-        <v>5371.0</v>
+        <v>5371</v>
       </c>
       <c r="K29" s="21">
-        <v>15001.0</v>
+        <v>15001</v>
       </c>
       <c r="L29" s="21">
-        <v>169596.0</v>
+        <v>169596</v>
       </c>
       <c r="M29" s="21">
         <v>77.03</v>
@@ -2052,18 +2054,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="23" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="24">
-        <v>3588.0</v>
+        <v>3588</v>
       </c>
       <c r="D30" s="21">
-        <v>10527.0</v>
+        <v>10527</v>
       </c>
       <c r="E30" s="24">
-        <v>121943.0</v>
+        <v>121943</v>
       </c>
       <c r="F30" s="21">
         <v>62.75</v>
@@ -2075,13 +2077,13 @@
         <v>43</v>
       </c>
       <c r="J30" s="21">
-        <v>3415.0</v>
+        <v>3415</v>
       </c>
       <c r="K30" s="21">
-        <v>9446.0</v>
+        <v>9446</v>
       </c>
       <c r="L30" s="21">
-        <v>138222.0</v>
+        <v>138222</v>
       </c>
       <c r="M30" s="21">
         <v>59.89</v>
@@ -2099,18 +2101,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="21" t="s">
         <v>45</v>
       </c>
       <c r="C31" s="22">
-        <v>3438.0</v>
+        <v>3438</v>
       </c>
       <c r="D31" s="21">
-        <v>10227.0</v>
+        <v>10227</v>
       </c>
       <c r="E31" s="22">
-        <v>135405.0</v>
+        <v>135405</v>
       </c>
       <c r="F31" s="21">
         <v>112.03</v>
@@ -2122,13 +2124,13 @@
         <v>45</v>
       </c>
       <c r="J31" s="21">
-        <v>3438.0</v>
+        <v>3438</v>
       </c>
       <c r="K31" s="21">
-        <v>10227.0</v>
+        <v>10227</v>
       </c>
       <c r="L31" s="21">
-        <v>135405.0</v>
+        <v>135405</v>
       </c>
       <c r="M31" s="21">
         <v>112.03</v>
@@ -2146,18 +2148,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="21" t="s">
         <v>43</v>
       </c>
       <c r="C32" s="22">
-        <v>3415.0</v>
+        <v>3415</v>
       </c>
       <c r="D32" s="21">
-        <v>9446.0</v>
+        <v>9446</v>
       </c>
       <c r="E32" s="22">
-        <v>138222.0</v>
+        <v>138222</v>
       </c>
       <c r="F32" s="21">
         <v>59.89</v>
@@ -2169,13 +2171,13 @@
         <v>42</v>
       </c>
       <c r="J32" s="21">
-        <v>3588.0</v>
+        <v>3588</v>
       </c>
       <c r="K32" s="21">
-        <v>10527.0</v>
+        <v>10527</v>
       </c>
       <c r="L32" s="21">
-        <v>121943.0</v>
+        <v>121943</v>
       </c>
       <c r="M32" s="21">
         <v>62.75</v>
@@ -2193,18 +2195,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="25" t="s">
         <v>46</v>
       </c>
       <c r="C33" s="24">
-        <v>2985.0</v>
+        <v>2985</v>
       </c>
       <c r="D33" s="21">
-        <v>9350.0</v>
+        <v>9350</v>
       </c>
       <c r="E33" s="24">
-        <v>79730.0</v>
+        <v>79730</v>
       </c>
       <c r="F33" s="21">
         <v>24.52</v>
@@ -2216,13 +2218,13 @@
         <v>47</v>
       </c>
       <c r="J33" s="26">
-        <v>1773.0</v>
+        <v>1773</v>
       </c>
       <c r="K33" s="26">
-        <v>3937.0</v>
+        <v>3937</v>
       </c>
       <c r="L33" s="26">
-        <v>90070.0</v>
+        <v>90070</v>
       </c>
       <c r="M33" s="26">
         <v>46.41</v>
@@ -2240,21 +2242,21 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="26" t="s">
         <v>48</v>
       </c>
       <c r="C34" s="27">
-        <v>1547.0</v>
+        <v>1547</v>
       </c>
       <c r="D34" s="26">
-        <v>3938.0</v>
+        <v>3938</v>
       </c>
       <c r="E34" s="27">
-        <v>53362.0</v>
+        <v>53362</v>
       </c>
       <c r="F34" s="26">
-        <v>38.55</v>
+        <v>38.549999999999997</v>
       </c>
       <c r="G34" s="26" t="b">
         <v>1</v>
@@ -2263,13 +2265,13 @@
         <v>46</v>
       </c>
       <c r="J34" s="26">
-        <v>2985.0</v>
+        <v>2985</v>
       </c>
       <c r="K34" s="26">
-        <v>9350.0</v>
+        <v>9350</v>
       </c>
       <c r="L34" s="26">
-        <v>79730.0</v>
+        <v>79730</v>
       </c>
       <c r="M34" s="26">
         <v>24.52</v>
@@ -2287,18 +2289,18 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="26" t="s">
         <v>47</v>
       </c>
       <c r="C35" s="27">
-        <v>1773.0</v>
+        <v>1773</v>
       </c>
       <c r="D35" s="26">
-        <v>3937.0</v>
+        <v>3937</v>
       </c>
       <c r="E35" s="27">
-        <v>90070.0</v>
+        <v>90070</v>
       </c>
       <c r="F35" s="26">
         <v>46.41</v>
@@ -2310,16 +2312,16 @@
         <v>48</v>
       </c>
       <c r="J35" s="29">
-        <v>1547.0</v>
+        <v>1547</v>
       </c>
       <c r="K35" s="29">
-        <v>3938.0</v>
+        <v>3938</v>
       </c>
       <c r="L35" s="29">
-        <v>53362.0</v>
+        <v>53362</v>
       </c>
       <c r="M35" s="29">
-        <v>38.55</v>
+        <v>38.549999999999997</v>
       </c>
       <c r="N35" s="29" t="b">
         <v>1</v>
@@ -2334,18 +2336,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="30" t="s">
         <v>50</v>
       </c>
       <c r="C36" s="31">
-        <v>1784.0</v>
+        <v>1784</v>
       </c>
       <c r="D36" s="26">
-        <v>3730.0</v>
+        <v>3730</v>
       </c>
       <c r="E36" s="31">
-        <v>45285.0</v>
+        <v>45285</v>
       </c>
       <c r="F36" s="26">
         <v>40.21</v>
@@ -2357,13 +2359,13 @@
         <v>50</v>
       </c>
       <c r="J36" s="29">
-        <v>1784.0</v>
+        <v>1784</v>
       </c>
       <c r="K36" s="29">
-        <v>3730.0</v>
+        <v>3730</v>
       </c>
       <c r="L36" s="29">
-        <v>45285.0</v>
+        <v>45285</v>
       </c>
       <c r="M36" s="29">
         <v>40.21</v>
@@ -2381,18 +2383,18 @@
         <v>51</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="32" t="s">
         <v>52</v>
       </c>
       <c r="C37" s="33">
-        <v>447.0</v>
+        <v>447</v>
       </c>
       <c r="D37" s="29">
-        <v>995.0</v>
+        <v>995</v>
       </c>
       <c r="E37" s="33">
-        <v>15684.0</v>
+        <v>15684</v>
       </c>
       <c r="F37" s="29">
         <v>12.94</v>
@@ -2404,13 +2406,13 @@
         <v>52</v>
       </c>
       <c r="J37" s="34">
-        <v>447.0</v>
+        <v>447</v>
       </c>
       <c r="K37" s="34">
-        <v>995.0</v>
+        <v>995</v>
       </c>
       <c r="L37" s="34">
-        <v>15684.0</v>
+        <v>15684</v>
       </c>
       <c r="M37" s="34">
         <v>12.94</v>
@@ -2428,8 +2430,8 @@
         <v>53</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="38" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
         <v>54</v>
       </c>
@@ -2461,19 +2463,19 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C40" s="5">
         <f>(E40+(D40*I51))/2</f>
-        <v>2595769.2</v>
+        <v>2599785</v>
       </c>
       <c r="D40" s="4">
-        <v>160632.0</v>
+        <v>160632</v>
       </c>
       <c r="E40" s="3">
-        <v>2468826.0</v>
+        <v>2468826</v>
       </c>
       <c r="F40" s="36" t="str">
         <f>IF(C40&lt;J47,I48,IF(C40&lt;J46,I47,IF(C40&lt;J45,I46,IF(C40&lt;J44,I45,IF(C40&lt;J43,I44,IF(C40&lt;J42,I43,IF(C40&lt;J41,I42,IF(C40&lt;J40,I41,I40))))))))</f>
@@ -2487,28 +2489,28 @@
       </c>
       <c r="J40" s="1">
         <f>((K40*I51)+L40)/2</f>
-        <v>823750</v>
+        <v>825000</v>
       </c>
       <c r="K40" s="35">
-        <v>50000.0</v>
+        <v>50000</v>
       </c>
       <c r="L40" s="35">
-        <v>800000.0</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="41" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C41" s="5">
         <f>(E41+(D41*I51))/2</f>
-        <v>2234218.9</v>
+        <v>2238035</v>
       </c>
       <c r="D41" s="4">
-        <v>152644.0</v>
+        <v>152644</v>
       </c>
       <c r="E41" s="5">
-        <v>1881122.0</v>
+        <v>1881122</v>
       </c>
       <c r="F41" s="36" t="str">
         <f>IF(C41&lt;J47,I48,IF(C41&lt;J46,I47,IF(C41&lt;J45,I46,IF(C41&lt;J44,I45,IF(C41&lt;J43,I44,IF(C41&lt;J42,I43,IF(C41&lt;J41,I42,IF(C41&lt;J40,I41,I40))))))))</f>
@@ -2522,28 +2524,28 @@
       </c>
       <c r="J41" s="1">
         <f>((K41*I51)+L41)/2</f>
-        <v>554250</v>
+        <v>555000</v>
       </c>
       <c r="K41" s="35">
-        <v>30000.0</v>
+        <v>30000</v>
       </c>
       <c r="L41" s="35">
-        <v>600000.0</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C42" s="5">
         <f>(E42+(D42*I51))/2</f>
-        <v>1962332.375</v>
+        <v>1965576.5</v>
       </c>
       <c r="D42" s="4">
-        <v>129765.0</v>
+        <v>129765</v>
       </c>
       <c r="E42" s="3">
-        <v>1725148.0</v>
+        <v>1725148</v>
       </c>
       <c r="F42" s="36" t="str">
         <f>IF(C42&lt;J47,I48,IF(C42&lt;J46,I47,IF(C42&lt;J45,I46,IF(C42&lt;J44,I45,IF(C42&lt;J43,I44,IF(C42&lt;J42,I43,IF(C42&lt;J41,I42,IF(C42&lt;J40,I41,I40))))))))</f>
@@ -2557,28 +2559,28 @@
       </c>
       <c r="J42" s="1">
         <f>((K42*I51)+L42)/2</f>
-        <v>344500</v>
+        <v>345000</v>
       </c>
       <c r="K42" s="35">
-        <v>20000.0</v>
+        <v>20000</v>
       </c>
       <c r="L42" s="35">
-        <v>350000.0</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="43" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C43" s="5">
         <f>(E43+(D43*I51))/2</f>
-        <v>1150945.225</v>
+        <v>1152912.5</v>
       </c>
       <c r="D43" s="4">
-        <v>78691.0</v>
+        <v>78691</v>
       </c>
       <c r="E43" s="6">
-        <v>968078.0</v>
+        <v>968078</v>
       </c>
       <c r="F43" s="36" t="str">
         <f>IF(C43&lt;J47,I48,IF(C43&lt;J46,I47,IF(C43&lt;J45,I46,IF(C43&lt;J44,I45,IF(C43&lt;J43,I44,IF(C43&lt;J42,I43,IF(C43&lt;J41,I42,IF(C43&lt;J40,I41,I40))))))))</f>
@@ -2592,28 +2594,28 @@
       </c>
       <c r="J43" s="1">
         <f>((K43*I51)+L43)/2</f>
-        <v>227125</v>
+        <v>227500</v>
       </c>
       <c r="K43" s="35">
-        <v>15000.0</v>
+        <v>15000</v>
       </c>
       <c r="L43" s="35">
-        <v>200000.0</v>
-      </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="44" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="5">
         <f>(E44+(D44*I51))/2</f>
-        <v>1296519.8</v>
+        <v>1298451</v>
       </c>
       <c r="D44" s="4">
-        <v>77248.0</v>
+        <v>77248</v>
       </c>
       <c r="E44" s="3">
-        <v>1283686.0</v>
+        <v>1283686</v>
       </c>
       <c r="F44" s="36" t="str">
         <f>IF(C44&lt;J47,I48,IF(C44&lt;J46,I47,IF(C44&lt;J45,I46,IF(C44&lt;J44,I45,IF(C44&lt;J43,I44,IF(C44&lt;J42,I43,IF(C44&lt;J41,I42,IF(C44&lt;J40,I41,I40))))))))</f>
@@ -2627,28 +2629,28 @@
       </c>
       <c r="J44" s="1">
         <f>((K44*I51)+L44)/2</f>
-        <v>126275</v>
+        <v>126500</v>
       </c>
       <c r="K44" s="35">
-        <v>9000.0</v>
+        <v>9000</v>
       </c>
       <c r="L44" s="35">
-        <v>100000.0</v>
-      </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="45" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C45" s="5">
         <f>(E45+(D45*I51))/2</f>
-        <v>1634852.7</v>
+        <v>1636760</v>
       </c>
       <c r="D45" s="4">
-        <v>76292.0</v>
+        <v>76292</v>
       </c>
       <c r="E45" s="3">
-        <v>1976556.0</v>
+        <v>1976556</v>
       </c>
       <c r="F45" s="36" t="str">
         <f>IF(C45&lt;J47,I48,IF(C45&lt;J46,I47,IF(C45&lt;J45,I46,IF(C45&lt;J44,I45,IF(C45&lt;J43,I44,IF(C45&lt;J42,I43,IF(C45&lt;J41,I42,IF(C45&lt;J40,I41,I40))))))))</f>
@@ -2662,28 +2664,28 @@
       </c>
       <c r="J45" s="1">
         <f>((K45*I51)+L45)/2</f>
-        <v>68900</v>
+        <v>69000</v>
       </c>
       <c r="K45" s="35">
-        <v>4000.0</v>
+        <v>4000</v>
       </c>
       <c r="L45" s="35">
-        <v>70000.0</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="46" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C46" s="5">
         <f>(E46+(D46*I51))/2</f>
-        <v>1089345.825</v>
+        <v>1091190.5</v>
       </c>
       <c r="D46" s="4">
-        <v>73787.0</v>
+        <v>73787</v>
       </c>
       <c r="E46" s="3">
-        <v>928002.0</v>
+        <v>928002</v>
       </c>
       <c r="F46" s="36" t="str">
         <f>IF(C46&lt;J47,I48,IF(C46&lt;J46,I47,IF(C46&lt;J45,I46,IF(C46&lt;J44,I45,IF(C46&lt;J43,I44,IF(C46&lt;J42,I43,IF(C46&lt;J41,I42,IF(C46&lt;J40,I41,I40))))))))</f>
@@ -2697,28 +2699,28 @@
       </c>
       <c r="J46" s="1">
         <f>((K46*I51)+L46)/2</f>
-        <v>45425</v>
+        <v>45500</v>
       </c>
       <c r="K46" s="35">
-        <v>3000.0</v>
+        <v>3000</v>
       </c>
       <c r="L46" s="35">
-        <v>40000.0</v>
-      </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="47" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C47" s="5">
         <f>(E47+(D47*I51))/2</f>
-        <v>1415227.675</v>
+        <v>1417060</v>
       </c>
       <c r="D47" s="4">
-        <v>73293.0</v>
+        <v>73293</v>
       </c>
       <c r="E47" s="3">
-        <v>1588139.0</v>
+        <v>1588139</v>
       </c>
       <c r="F47" s="36" t="str">
         <f>IF(C47&lt;J47,I48,IF(C47&lt;J46,I47,IF(C47&lt;J45,I46,IF(C47&lt;J44,I45,IF(C47&lt;J43,I44,IF(C47&lt;J42,I43,IF(C47&lt;J41,I42,IF(C47&lt;J40,I41,I40))))))))</f>
@@ -2732,28 +2734,28 @@
       </c>
       <c r="J47" s="1">
         <f>((K47*I51)+L47)/2</f>
-        <v>26950</v>
+        <v>27000</v>
       </c>
       <c r="K47" s="35">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="L47" s="35">
-        <v>20000.0</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="48" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C48" s="37">
         <f>(E48+(D48*I51))/2</f>
-        <v>913741.475</v>
+        <v>915447</v>
       </c>
       <c r="D48" s="9">
-        <v>68221.0</v>
+        <v>68221</v>
       </c>
       <c r="E48" s="8">
-        <v>671137.0</v>
+        <v>671137</v>
       </c>
       <c r="F48" s="38" t="s">
         <v>19</v>
@@ -2769,25 +2771,25 @@
         <v>0</v>
       </c>
       <c r="K48" s="35">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="L48" s="35">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C49" s="5">
         <f>(E49+(D49*I51))/2</f>
-        <v>1004700.35</v>
+        <v>1006376.5</v>
       </c>
       <c r="D49" s="4">
-        <v>67046.0</v>
+        <v>67046</v>
       </c>
       <c r="E49" s="3">
-        <v>872971.0</v>
+        <v>872971</v>
       </c>
       <c r="F49" s="36" t="str">
         <f>IF(C49&lt;J47,I48,IF(C49&lt;J46,I47,IF(C49&lt;J45,I46,IF(C49&lt;J44,I45,IF(C49&lt;J43,I44,IF(C49&lt;J42,I43,IF(C49&lt;J41,I42,IF(C49&lt;J40,I41,I40))))))))</f>
@@ -2797,19 +2799,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="11" t="s">
         <v>22</v>
       </c>
       <c r="C50" s="39">
         <f>(E50+(D50*I51))/2</f>
-        <v>590826.65</v>
+        <v>592097.5</v>
       </c>
       <c r="D50" s="10">
-        <v>50834.0</v>
+        <v>50834</v>
       </c>
       <c r="E50" s="12">
-        <v>320017.0</v>
+        <v>320017</v>
       </c>
       <c r="F50" s="40" t="str">
         <f>IF(C50&lt;J47,I48,IF(C50&lt;J46,I47,IF(C50&lt;J45,I46,IF(C50&lt;J44,I45,IF(C50&lt;J43,I44,IF(C50&lt;J42,I43,IF(C50&lt;J41,I42,IF(C50&lt;J40,I41,I40))))))))</f>
@@ -2822,19 +2824,19 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C51" s="39">
         <f>(E51+(D51*I51))/2</f>
-        <v>565315.825</v>
+        <v>566257.5</v>
       </c>
       <c r="D51" s="10">
-        <v>37667.0</v>
+        <v>37667</v>
       </c>
       <c r="E51" s="12">
-        <v>492176.0</v>
+        <v>492176</v>
       </c>
       <c r="F51" s="40" t="str">
         <f>IF(C51&lt;J47,I48,IF(C51&lt;J46,I47,IF(C51&lt;J45,I46,IF(C51&lt;J44,I45,IF(C51&lt;J43,I44,IF(C51&lt;J42,I43,IF(C51&lt;J41,I42,IF(C51&lt;J40,I41,I40))))))))</f>
@@ -2844,22 +2846,22 @@
         <v>0</v>
       </c>
       <c r="I51" s="35">
-        <v>16.95</v>
-      </c>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C52" s="39">
         <f>(E52+(D52*I51))/2</f>
-        <v>555154.6</v>
+        <v>556074</v>
       </c>
       <c r="D52" s="10">
-        <v>36776.0</v>
+        <v>36776</v>
       </c>
       <c r="E52" s="12">
-        <v>486956.0</v>
+        <v>486956</v>
       </c>
       <c r="F52" s="40" t="str">
         <f>IF(C52&lt;J47,I48,IF(C52&lt;J46,I47,IF(C52&lt;J45,I46,IF(C52&lt;J44,I45,IF(C52&lt;J43,I44,IF(C52&lt;J42,I43,IF(C52&lt;J41,I42,IF(C52&lt;J40,I41,I40))))))))</f>
@@ -2869,19 +2871,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C53" s="41">
         <f>(E53+(D53*I51))/2</f>
-        <v>467023</v>
+        <v>467896.5</v>
       </c>
       <c r="D53" s="13">
-        <v>34940.0</v>
+        <v>34940</v>
       </c>
       <c r="E53" s="42">
-        <v>341813.0</v>
+        <v>341813</v>
       </c>
       <c r="F53" s="43" t="str">
         <f>IF(C53&lt;J47,I48,IF(C53&lt;J46,I47,IF(C53&lt;J45,I46,IF(C53&lt;J44,I45,IF(C53&lt;J43,I44,IF(C53&lt;J42,I43,IF(C53&lt;J41,I42,IF(C53&lt;J40,I41,I40))))))))</f>
@@ -2897,19 +2899,19 @@
       <c r="K53" s="35"/>
       <c r="L53" s="35"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C54" s="41">
         <f>(E54+(D54*I51))/2</f>
-        <v>444619.425</v>
+        <v>445337</v>
       </c>
       <c r="D54" s="13">
-        <v>28703.0</v>
+        <v>28703</v>
       </c>
       <c r="E54" s="16">
-        <v>402723.0</v>
+        <v>402723</v>
       </c>
       <c r="F54" s="43" t="str">
         <f>IF(C54&lt;J47,I48,IF(C54&lt;J46,I47,IF(C54&lt;J45,I46,IF(C54&lt;J44,I45,IF(C54&lt;J43,I44,IF(C54&lt;J42,I43,IF(C54&lt;J41,I42,IF(C54&lt;J40,I41,I40))))))))</f>
@@ -2931,19 +2933,19 @@
         <v>66</v>
       </c>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="15" t="s">
         <v>30</v>
       </c>
       <c r="C55" s="41">
         <f>(E55+(D55*I51))/2</f>
-        <v>415708.8</v>
+        <v>416390.5</v>
       </c>
       <c r="D55" s="13">
-        <v>27268.0</v>
+        <v>27268</v>
       </c>
       <c r="E55" s="16">
-        <v>369225.0</v>
+        <v>369225</v>
       </c>
       <c r="F55" s="43" t="str">
         <f>IF(C55&lt;J47,I48,IF(C55&lt;J46,I47,IF(C55&lt;J45,I46,IF(C55&lt;J44,I45,IF(C55&lt;J43,I44,IF(C55&lt;J42,I43,IF(C55&lt;J41,I42,IF(C55&lt;J40,I41,I40))))))))</f>
@@ -2958,28 +2960,28 @@
       </c>
       <c r="J55" s="1">
         <f>(L55+(K55*I51))/2</f>
-        <v>227293.45</v>
+        <v>227560</v>
       </c>
       <c r="K55" s="35">
-        <v>10662.0</v>
+        <v>10662</v>
       </c>
       <c r="L55" s="35">
-        <v>273866.0</v>
-      </c>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
+        <v>273866</v>
+      </c>
+    </row>
+    <row r="56" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C56" s="41">
         <f>(E56+(D56*I51))/2</f>
-        <v>405317.925</v>
+        <v>405990.5</v>
       </c>
       <c r="D56" s="13">
-        <v>26903.0</v>
+        <v>26903</v>
       </c>
       <c r="E56" s="16">
-        <v>354630.0</v>
+        <v>354630</v>
       </c>
       <c r="F56" s="43" t="str">
         <f>IF(C56&lt;J47,I48,IF(C56&lt;J46,I47,IF(C50&lt;J45,I46,IF(C56&lt;J44,I45,IF(C56&lt;J43,I44,IF(C56&lt;J42,I43,IF(C56&lt;J41,I42,IF(C56&lt;J40,I41,I40))))))))</f>
@@ -2989,19 +2991,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="15" t="s">
         <v>33</v>
       </c>
       <c r="C57" s="41">
         <f>(E57+(D57*I51))/2</f>
-        <v>359639.05</v>
+        <v>360296</v>
       </c>
       <c r="D57" s="13">
-        <v>26278.0</v>
+        <v>26278</v>
       </c>
       <c r="E57" s="16">
-        <v>273866.0</v>
+        <v>273866</v>
       </c>
       <c r="F57" s="43" t="str">
         <f>IF(C57&lt;J47,I48,IF(C57&lt;J46,I47,IF(C57&lt;J45,I46,IF(C57&lt;J44,I45,IF(C57&lt;J43,I44,IF(C57&lt;J42,I43,IF(C57&lt;J41,I42,IF(C57&lt;J40,I41,I40))))))))</f>
@@ -3011,19 +3013,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C58" s="41">
         <f>(E58+(D58*I51))/2</f>
-        <v>391712.375</v>
+        <v>392365.5</v>
       </c>
       <c r="D58" s="13">
-        <v>26125.0</v>
+        <v>26125</v>
       </c>
       <c r="E58" s="16">
-        <v>340606.0</v>
+        <v>340606</v>
       </c>
       <c r="F58" s="43" t="str">
         <f>IF(C58&lt;J47,I48,IF(C58&lt;J46,I47,IF(C58&lt;J45,I46,IF(C58&lt;J44,I45,IF(C58&lt;J43,I44,IF(C58&lt;J42,I43,IF(C58&lt;J41,I42,IF(C58&lt;J40,I41,I40))))))))</f>
@@ -3033,19 +3035,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="15" t="s">
         <v>35</v>
       </c>
       <c r="C59" s="41">
         <f>(E59+(D59*I51))/2</f>
-        <v>345916.8</v>
+        <v>346552.5</v>
       </c>
       <c r="D59" s="13">
-        <v>25428.0</v>
+        <v>25428</v>
       </c>
       <c r="E59" s="16">
-        <v>260829.0</v>
+        <v>260829</v>
       </c>
       <c r="F59" s="43" t="str">
         <f>IF(C59&lt;J47,I48,IF(C59&lt;J46,I47,IF(C59&lt;J45,I46,IF(C59&lt;J44,I45,IF(C59&lt;J43,I44,IF(C59&lt;J42,I43,IF(C59&lt;J41,I42,IF(C59&lt;J40,I41,I40))))))))</f>
@@ -3055,19 +3057,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="17" t="s">
         <v>36</v>
       </c>
       <c r="C60" s="44">
         <f>(E60+(D60*I51))/2</f>
-        <v>325895.55</v>
+        <v>326362.5</v>
       </c>
       <c r="D60" s="17">
-        <v>18678.0</v>
+        <v>18678</v>
       </c>
       <c r="E60" s="18">
-        <v>335199.0</v>
+        <v>335199</v>
       </c>
       <c r="F60" s="45" t="str">
         <f>IF(C60&lt;J47,I48,IF(C60&lt;J46,I47,IF(C60&lt;J45,I46,IF(C60&lt;J44,I45,IF(C60&lt;J43,I44,IF(C60&lt;J42,I43,IF(C60&lt;J41,I42,IF(C60&lt;J40,I41,I40))))))))</f>
@@ -3077,19 +3079,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="17" t="s">
         <v>37</v>
       </c>
       <c r="C61" s="44">
         <f>(E61+(D61*I51))/2</f>
-        <v>239640.8</v>
+        <v>240088</v>
       </c>
       <c r="D61" s="17">
-        <v>17888.0</v>
+        <v>17888</v>
       </c>
       <c r="E61" s="18">
-        <v>176080.0</v>
+        <v>176080</v>
       </c>
       <c r="F61" s="45" t="str">
         <f>IF(C61&lt;J47,I48,IF(C61&lt;J46,I47,IF(C61&lt;J45,I46,IF(C61&lt;J44,I45,IF(C61&lt;J43,I44,IF(C61&lt;J42,I43,IF(C61&lt;J41,I42,IF(C61&lt;J40,I41,I40))))))))</f>
@@ -3099,19 +3101,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="15" t="s">
         <v>20</v>
       </c>
       <c r="C62" s="41">
         <f>(E62+(D62*I51))/2</f>
-        <v>494974.725</v>
+        <v>495389.5</v>
       </c>
       <c r="D62" s="13">
-        <v>16591.0</v>
+        <v>16591</v>
       </c>
       <c r="E62" s="16">
-        <v>708732.0</v>
+        <v>708732</v>
       </c>
       <c r="F62" s="43" t="str">
         <f>IF(C62&lt;J47,I48,IF(C62&lt;J46,I47,IF(C62&lt;J45,I46,IF(C62&lt;J44,I45,IF(C62&lt;J43,I44,IF(C62&lt;J42,I43,IF(C62&lt;J41,I42,IF(C62&lt;J40,I41,I40))))))))</f>
@@ -3121,19 +3123,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="17" t="s">
         <v>38</v>
       </c>
       <c r="C63" s="44">
         <f>(E63+(D63*I51))/2</f>
-        <v>246256.875</v>
+        <v>246641</v>
       </c>
       <c r="D63" s="17">
-        <v>15365.0</v>
+        <v>15365</v>
       </c>
       <c r="E63" s="18">
-        <v>232077.0</v>
+        <v>232077</v>
       </c>
       <c r="F63" s="45" t="str">
         <f>IF(C63&lt;J47,I48,IF(C63&lt;J46,I47,IF(C63&lt;J45,I46,IF(C63&lt;J44,I45,IF(C63&lt;J43,I44,IF(C63&lt;J42,I43,IF(C63&lt;J41,I42,IF(C63&lt;J40,I41,I40))))))))</f>
@@ -3143,19 +3145,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="21" t="s">
         <v>39</v>
       </c>
       <c r="C64" s="46">
         <f>(E64+(D64*I51))/2</f>
-        <v>211931.475</v>
+        <v>212306.5</v>
       </c>
       <c r="D64" s="21">
-        <v>15001.0</v>
+        <v>15001</v>
       </c>
       <c r="E64" s="22">
-        <v>169596.0</v>
+        <v>169596</v>
       </c>
       <c r="F64" s="47" t="str">
         <f>IF(C64&lt;J47,I48,IF(C64&lt;J46,I47,IF(C64&lt;J45,I46,IF(C64&lt;J44,I45,IF(C64&lt;J43,I44,IF(C64&lt;J42,I43,IF(C64&lt;J41,I42,IF(C64&lt;J40,I41,I40))))))))</f>
@@ -3165,19 +3167,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="17" t="s">
         <v>28</v>
       </c>
       <c r="C65" s="44">
         <f>(E65+(D65*I51))/2</f>
-        <v>337746.85</v>
+        <v>338119.5</v>
       </c>
       <c r="D65" s="17">
-        <v>14906.0</v>
+        <v>14906</v>
       </c>
       <c r="E65" s="18">
-        <v>422837.0</v>
+        <v>422837</v>
       </c>
       <c r="F65" s="45" t="str">
         <f>IF(C65&lt;J47,I48,IF(C65&lt;J46,I47,IF(C65&lt;J45,I46,IF(C65&lt;J44,I45,IF(C65&lt;J43,I44,IF(C65&lt;J42,I43,IF(C65&lt;J41,I42,IF(C65&lt;J40,I41,I40))))))))</f>
@@ -3187,19 +3189,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="21" t="s">
         <v>41</v>
       </c>
       <c r="C66" s="46">
         <f>(E66+(D66*I51))/2</f>
-        <v>194430.375</v>
+        <v>194739.5</v>
       </c>
       <c r="D66" s="21">
-        <v>12365.0</v>
+        <v>12365</v>
       </c>
       <c r="E66" s="22">
-        <v>179274.0</v>
+        <v>179274</v>
       </c>
       <c r="F66" s="47" t="str">
         <f>IF(C66&lt;J47,I48,IF(C66&lt;J46,I47,IF(C66&lt;J45,I46,IF(C66&lt;J44,I45,IF(C66&lt;J43,I44,IF(C66&lt;J42,I43,IF(C66&lt;J41,I42,IF(C66&lt;J40,I41,I40))))))))</f>
@@ -3209,19 +3211,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="23" t="s">
         <v>40</v>
       </c>
       <c r="C67" s="46">
         <f>(E67+(D67*I51))/2</f>
-        <v>198349.075</v>
+        <v>198657.5</v>
       </c>
       <c r="D67" s="21">
-        <v>12337.0</v>
+        <v>12337</v>
       </c>
       <c r="E67" s="24">
-        <v>187586.0</v>
+        <v>187586</v>
       </c>
       <c r="F67" s="47" t="str">
         <f>IF(C67&lt;J47,I48,IF(C67&lt;J46,I47,IF(C67&lt;J45,I46,IF(C67&lt;J44,I45,IF(C67&lt;J43,I44,IF(C67&lt;J42,I43,IF(C67&lt;J41,I42,IF(C67&lt;J40,I41,I40))))))))</f>
@@ -3231,19 +3233,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="23" t="s">
         <v>42</v>
       </c>
       <c r="C68" s="46">
         <f>(E68+(D68*I51))/2</f>
-        <v>150187.825</v>
+        <v>150451</v>
       </c>
       <c r="D68" s="21">
-        <v>10527.0</v>
+        <v>10527</v>
       </c>
       <c r="E68" s="24">
-        <v>121943.0</v>
+        <v>121943</v>
       </c>
       <c r="F68" s="47" t="str">
         <f>IF(C68&lt;J47,I48,IF(C68&lt;J46,I47,IF(C68&lt;J45,I46,IF(C68&lt;J44,I45,IF(C68&lt;J43,I44,IF(C68&lt;J42,I43,IF(C68&lt;J41,I42,IF(C68&lt;J40,I41,I40))))))))</f>
@@ -3253,19 +3255,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="21" t="s">
         <v>45</v>
       </c>
       <c r="C69" s="46">
         <f>(E69+(D69*I51))/2</f>
-        <v>154376.325</v>
+        <v>154632</v>
       </c>
       <c r="D69" s="21">
-        <v>10227.0</v>
+        <v>10227</v>
       </c>
       <c r="E69" s="22">
-        <v>135405.0</v>
+        <v>135405</v>
       </c>
       <c r="F69" s="47" t="str">
         <f>IF(C69&lt;J47,I48,IF(C69&lt;J46,I47,IF(C69&lt;J45,I46,IF(C69&lt;J44,I45,IF(C69&lt;J43,I44,IF(C69&lt;J42,I43,IF(C69&lt;J41,I42,IF(C69&lt;J40,I41,I40))))))))</f>
@@ -3275,19 +3277,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="21" t="s">
         <v>43</v>
       </c>
       <c r="C70" s="46">
         <f>(E70+(D70*I51))/2</f>
-        <v>149165.85</v>
+        <v>149402</v>
       </c>
       <c r="D70" s="21">
-        <v>9446.0</v>
+        <v>9446</v>
       </c>
       <c r="E70" s="22">
-        <v>138222.0</v>
+        <v>138222</v>
       </c>
       <c r="F70" s="47" t="str">
         <f>IF(C70&lt;J47,I48,IF(C70&lt;J46,I47,IF(C70&lt;J45,I46,IF(C70&lt;J44,I45,IF(C70&lt;J43,I44,IF(C70&lt;J42,I43,IF(C70&lt;J41,I42,IF(C70&lt;J40,I41,I40))))))))</f>
@@ -3297,19 +3299,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="30" t="s">
         <v>46</v>
       </c>
       <c r="C71" s="48">
         <f>(E71+(D71*I51))/2</f>
-        <v>119106.25</v>
+        <v>119340</v>
       </c>
       <c r="D71" s="26">
-        <v>9350.0</v>
+        <v>9350</v>
       </c>
       <c r="E71" s="31">
-        <v>79730.0</v>
+        <v>79730</v>
       </c>
       <c r="F71" s="49" t="str">
         <f>IF(C71&lt;J47,I48,IF(C71&lt;J46,I47,IF(C71&lt;J45,I46,IF(C71&lt;J44,I45,IF(C71&lt;J43,I44,IF(C71&lt;J42,I43,IF(C71&lt;J41,I42,IF(C71&lt;J40,I41,I40))))))))</f>
@@ -3319,19 +3321,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="29" t="s">
         <v>48</v>
       </c>
       <c r="C72" s="50">
         <f>(E72+(D72*I51))/2</f>
-        <v>60055.55</v>
+        <v>60154</v>
       </c>
       <c r="D72" s="29">
-        <v>3938.0</v>
+        <v>3938</v>
       </c>
       <c r="E72" s="51">
-        <v>53362.0</v>
+        <v>53362</v>
       </c>
       <c r="F72" s="52" t="str">
         <f>IF(C72&lt;J47,I48,IF(C72&lt;J46,I47,IF(C72&lt;J45,I46,IF(C72&lt;J44,I45,IF(C72&lt;J43,I44,IF(C72&lt;J42,I43,IF(C72&lt;J41,I42,IF(C72&lt;J40,I41,I40))))))))</f>
@@ -3341,19 +3343,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="26" t="s">
         <v>47</v>
       </c>
       <c r="C73" s="48">
         <f>(E73+(D73*I51))/2</f>
-        <v>78401.075</v>
+        <v>78499.5</v>
       </c>
       <c r="D73" s="26">
-        <v>3937.0</v>
+        <v>3937</v>
       </c>
       <c r="E73" s="27">
-        <v>90070.0</v>
+        <v>90070</v>
       </c>
       <c r="F73" s="49" t="str">
         <f>IF(C73&lt;J47,I48,IF(C73&lt;J46,I47,IF(C73&lt;J45,I46,IF(C73&lt;J44,I45,IF(C73&lt;J43,I44,IF(C73&lt;J42,I43,IF(C73&lt;J41,I42,IF(C73&lt;J40,I41,I40))))))))</f>
@@ -3363,19 +3365,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="32" t="s">
         <v>50</v>
       </c>
       <c r="C74" s="50">
         <f>(E74+(D74*I51))/2</f>
-        <v>54254.25</v>
+        <v>54347.5</v>
       </c>
       <c r="D74" s="29">
-        <v>3730.0</v>
+        <v>3730</v>
       </c>
       <c r="E74" s="33">
-        <v>45285.0</v>
+        <v>45285</v>
       </c>
       <c r="F74" s="52" t="str">
         <f>IF(C74&lt;J47,I48,IF(C74&lt;J46,I47,IF(C74&lt;J45,I46,IF(C74&lt;J44,I45,IF(C74&lt;J43,I44,IF(C74&lt;J42,I43,IF(C74&lt;J41,I42,IF(C74&lt;J40,I41,I40))))))))</f>
@@ -3385,19 +3387,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="53" t="s">
         <v>52</v>
       </c>
       <c r="C75" s="54">
         <f>(E75+(D75*I51))/2</f>
-        <v>16274.625</v>
+        <v>16299.5</v>
       </c>
       <c r="D75" s="34">
-        <v>995.0</v>
+        <v>995</v>
       </c>
       <c r="E75" s="55">
-        <v>15684.0</v>
+        <v>15684</v>
       </c>
       <c r="F75" s="56" t="str">
         <f>IF(C75&lt;J47,I48,IF(C75&lt;J46,I47,IF(C75&lt;J45,I46,IF(C75&lt;J44,I45,IF(C75&lt;J43,I44,IF(C75&lt;J42,I43,IF(C75&lt;J41,I42,IF(C75&lt;J40,I41,I40))))))))</f>
@@ -3407,935 +3409,933 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="76" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>